<commit_message>
Stage 8 review fixes: B-027
</commit_message>
<xml_diff>
--- a/output/archive/BrindlewytheData/Studies/2025/BW25_0231/Run_sheets/BW25_0231_RUN04.xlsx
+++ b/output/archive/BrindlewytheData/Studies/2025/BW25_0231/Run_sheets/BW25_0231_RUN04.xlsx
@@ -169,7 +169,7 @@
   <commentList>
     <comment ref="B13" authorId="0" shapeId="0">
       <text>
-        <t>Confirm the top concentration against the study plan before the set is released</t>
+        <t>Use the sample cards for test-lot and solvent records.</t>
       </text>
     </comment>
   </commentList>
@@ -179,12 +179,12 @@
 <file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>Jason Scanlon</author>
+    <author>Ravi Deshmukh</author>
   </authors>
   <commentList>
-    <comment ref="D6" authorId="0" shapeId="0">
+    <comment ref="C6" authorId="0" shapeId="0">
       <text>
-        <t>Plate 3 baseline drifted early in the run. Stéphane to confirm the cell batch before we accept the plate.</t>
+        <t>TP04-02866 is solubility-limited; retain its qualification when quoting the result.</t>
       </text>
     </comment>
   </commentList>
@@ -199,7 +199,7 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>Compound 02716 cell 2 is noisy. Keep it in the table and flag it in the report.</t>
+        <t>TP04-02866 carries the solubility qualification. TP04-02716 has no QC flag in the result table.</t>
       </text>
     </comment>
   </commentList>
@@ -505,7 +505,8 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BW25_0231 run sheet 04: hERG automated patch clamp</t>
+          <t>Brindlewythe Biosciences Ltd, a Tarnovell company
+BW25_0231 run sheet 04: hERG automated patch clamp</t>
         </is>
       </c>
     </row>
@@ -580,12 +581,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Runs</t>
+          <t>Study start / completion</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>06/06/2025 to 24/06/2025</t>
+          <t>06/06/2025 / 25/06/2025</t>
         </is>
       </c>
     </row>
@@ -654,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -678,7 +679,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Acceptance</t>
+          <t>Acceptance / interpretation</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -688,7 +689,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Record</t>
         </is>
       </c>
     </row>
@@ -700,7 +701,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Within historical range</t>
+          <t>5–50 nM</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
@@ -715,81 +716,81 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Seal resistance</t>
+          <t>Cell quality</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Above plate minimum</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
+          <t>Consult original cell records</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>See compound QC notes</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Original run sheets</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Vehicle current run-down</t>
+          <t>Concentration response</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Within 10% across the run</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
+          <t>6-point, 3-fold dilution</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Top concentration in run sheet</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Original run sheets</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Plate 3 vehicle baseline</t>
+          <t>Solubility qualification</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Within 10% across the run</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr"/>
+          <t>Use highest evaluable concentration</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>See compound QC notes</t>
+        </is>
+      </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Hold</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Reference compound on each plate</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Present on every plate</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Accepted</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Plates accepted</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
+          <t>hERG IC50 table</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Final tables</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Plate-level audit trail retained in original run sheets</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -820,14 +821,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>hERG IC50, automated patch clamp, 32 compounds</t>
+          <t>hERG IC50, automated patch clamp: 32 compounds</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Values marked &gt; were censored at the top concentration. Where one cell was discarded the geomean uses the remaining cells; see the QC note column.</t>
+          <t>Compound IC50 is the geometric mean of finite cell IC50s only when finite values form a majority of accepted cells. Otherwise retain the censored value, using the highest evaluable concentration for solubility-limited records. Blank cell fields do not by themselves indicate exclusion.</t>
         </is>
       </c>
     </row>

</xml_diff>